<commit_message>
More on OL accruals
</commit_message>
<xml_diff>
--- a/data/obx_xlsx/AFK.OL.xlsx
+++ b/data/obx_xlsx/AFK.OL.xlsx
@@ -11586,15 +11586,17 @@
       <c r="O27" s="14">
         <v>742.52</v>
       </c>
-      <c r="P27" s="16"/>
+      <c r="P27" s="14">
+        <v>613.22</v>
+      </c>
       <c r="Q27" s="14">
         <v>318.0</v>
       </c>
-      <c r="R27" s="16">
-        <v>0.0</v>
-      </c>
-      <c r="S27" s="15">
-        <v>0.08</v>
+      <c r="R27" s="14">
+        <v>311.65</v>
+      </c>
+      <c r="S27" s="14">
+        <v>212.02</v>
       </c>
       <c r="T27" s="14">
         <v>131.66</v>
@@ -13458,13 +13460,33 @@
       <c r="P68" s="14">
         <v>812.56</v>
       </c>
-      <c r="Q68" s="16"/>
-      <c r="R68" s="16"/>
-      <c r="S68" s="16"/>
-      <c r="T68" s="16"/>
-      <c r="U68" s="16"/>
-      <c r="V68" s="16"/>
-      <c r="W68" s="16"/>
+      <c r="Q68" s="14">
+        <v>1043.2</v>
+      </c>
+      <c r="R68" s="16">
+        <f t="shared" ref="R68:W68" si="1">SUM(R69,R72,R79,R87,R94)</f>
+        <v>385.93</v>
+      </c>
+      <c r="S68" s="16">
+        <f t="shared" si="1"/>
+        <v>377.99</v>
+      </c>
+      <c r="T68" s="16">
+        <f t="shared" si="1"/>
+        <v>79</v>
+      </c>
+      <c r="U68" s="16">
+        <f t="shared" si="1"/>
+        <v>37.28</v>
+      </c>
+      <c r="V68" s="16">
+        <f t="shared" si="1"/>
+        <v>37.66</v>
+      </c>
+      <c r="W68" s="16">
+        <f t="shared" si="1"/>
+        <v>42.57</v>
+      </c>
     </row>
     <row r="69" ht="15.0" customHeight="1">
       <c r="A69" s="13" t="s">

</xml_diff>